<commit_message>
feat(minigame): add vending roulette on the GateDrop mechanic
- GateDrop mechanic (Content/Minigame/GateDrop): a can bounces down a
  peg board, buttons open the gate above each outlet, the outlet decides
  the outcome. Board fits the stage resolution; temp pixel art and
  procedural sound are generated at runtime.
- vending_roulette on the Plaza DrinkMachine: 5 drinks + dud drink
  (Item rows 2-7), new rail node RailNode_A8, no start condition.
- Framework: SourceBounds placement (MinigameProjection) opens the window
  over the source and follows it on LowResPixelRenderer.OnViewUpdated;
  MinigameBase.OnBind and CanAbort hooks; HUD hint hidden while a
  blocking page is open.
- Tests: GateDropBoard, GateDropLayout, MinigameProjection, PixelCanvas
  (EditMode 276/276 pass).
- Docs: Docs/Minigames/ design docs (README, templates, vending roulette,
  GateDrop format), framework section 12, roadmap, session log.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Item.xlsx
+++ b/Table/Excel/Item.xlsx
@@ -1,97 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TokTak\Desktop\Local\Unity\LOTW\LOTW\Table\Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27954D78-C9BF-4D64-B54F-17E0C7D87B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{35518A88-0317-48A7-9E0F-C9981C476B9C}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Item" sheetId="1" r:id="rId1"/>
+    <sheet name="Item" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
-  <si>
-    <t>DataId</t>
-  </si>
-  <si>
-    <t>ItemId</t>
-  </si>
-  <si>
-    <t>DisplayName</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Icon</t>
-  </si>
-  <si>
-    <t>MaxStack</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>rose</t>
-  </si>
-  <si>
-    <t>@item.rose.name</t>
-  </si>
-  <si>
-    <t>@item.rose.desc</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color rgb="FF808080"/>
       <sz val="11"/>
-      <color rgb="FF808080"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -107,20 +59,22 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -143,27 +97,87 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EDE1D533-195C-433F-93DA-44E8B5A38EF4}" name="Item" displayName="Item" ref="B2:G4" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="B2:G4" xr:uid="{EDE1D533-195C-433F-93DA-44E8B5A38EF4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Item" displayName="Item" ref="B2:G10" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:G10"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0CEF135A-7C6A-4058-B43F-3893FC2AEBD6}" name="DataId"/>
-    <tableColumn id="2" xr3:uid="{2B3C629D-6877-48BF-859C-B96F10DBAA4D}" name="ItemId" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{75FB7605-B48E-434B-B845-C688E83ECBF4}" name="DisplayName" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{1F4D0055-347C-4927-B405-CDC1DDCFE2A5}" name="Description" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{061A01EB-5EF4-4D68-80A8-120D62CF9241}" name="Icon" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{7C5CEC00-8932-4FDC-A01E-F3E67DF23E17}" name="MaxStack"/>
+    <tableColumn id="1" name="DataId"/>
+    <tableColumn id="2" name="ItemId" dataDxfId="4"/>
+    <tableColumn id="3" name="DisplayName" dataDxfId="3"/>
+    <tableColumn id="4" name="Description" dataDxfId="2"/>
+    <tableColumn id="5" name="Icon" dataDxfId="1"/>
+    <tableColumn id="6" name="MaxStack"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -465,81 +479,259 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD1E2E40-A28E-4B47-B3DD-72519159B69A}">
-  <dimension ref="B2:G4"/>
-  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.125" customWidth="1"/>
-    <col min="2" max="2" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.125" bestFit="1" customWidth="1"/>
+    <col width="3.125" customWidth="1" style="3" min="1" max="1"/>
+    <col width="9.625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="9.625" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
+    <col width="16.75" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
+    <col width="15.625" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
+    <col width="7.5" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
+    <col width="12.125" bestFit="1" customWidth="1" style="3" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
+    <row r="2" ht="16.5" customHeight="1" s="3">
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>DataId</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>ItemId</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>DisplayName</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>MaxStack</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="3">
+      <c r="B4" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>@item.rose.name</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>@item.rose.desc</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="0" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>drink_soda</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_soda.name</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_soda.desc</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>drink_milk</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_milk.name</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_milk.desc</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="n">
         <v>4</v>
       </c>
-      <c r="G2" t="s">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>drink_coffee</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_coffee.name</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_coffee.desc</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>drink_lemon</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_lemon.name</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_lemon.desc</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="n">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>drink_greentea</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_greentea.name</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_greentea.desc</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>drink_dud</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_dud.name</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>@item.drink_dud.desc</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" t="n">
         <v>99</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>